<commit_message>
Báo giá BG-2026/002: bổ sung dây điện Cu/PVC 1x4 (15.331 x 1,1)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
+++ b/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
@@ -11,7 +11,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Báo giá'!$19:$19</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Báo giá'!$A$1:$G$42</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Báo giá'!$A$1:$G$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -761,7 +761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.5" customWidth="1" min="1" max="1"/>
@@ -1131,7 +1131,7 @@
       </c>
       <c r="B21" s="24" t="inlineStr">
         <is>
-          <t>Dây điện ô van Cu/PVC/PVC 2×2.5mm² – 300/500V</t>
+          <t>Dây điện Cu/PVC 1×4mm²</t>
         </is>
       </c>
       <c r="C21" s="23" t="inlineStr">
@@ -1139,94 +1139,109 @@
           <t>m</t>
         </is>
       </c>
-      <c r="D21" s="25" t="n">
-        <v>1400</v>
-      </c>
+      <c r="D21" s="25" t="n"/>
       <c r="E21" s="25" t="n">
-        <v>24096</v>
+        <v>16864</v>
       </c>
       <c r="F21" s="26">
         <f>IF(OR(D21="",E21=""),"",ROUND(D21*E21,0))</f>
         <v/>
       </c>
-      <c r="G21" s="27" t="inlineStr"/>
-    </row>
-    <row r="22" ht="20" customHeight="1">
-      <c r="A22" s="28" t="inlineStr">
+      <c r="G21" s="27" t="inlineStr">
+        <is>
+          <t>Chờ số lượng</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="19" customHeight="1">
+      <c r="A22" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="B22" s="19" t="inlineStr">
+        <is>
+          <t>Dây điện ô van Cu/PVC/PVC 2×2.5mm² – 300/500V</t>
+        </is>
+      </c>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D22" s="20" t="n">
+        <v>1400</v>
+      </c>
+      <c r="E22" s="20" t="n">
+        <v>24096</v>
+      </c>
+      <c r="F22" s="21">
+        <f>IF(OR(D22="",E22=""),"",ROUND(D22*E22,0))</f>
+        <v/>
+      </c>
+      <c r="G22" s="22" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="28" t="inlineStr">
         <is>
           <t>Cộng tiền hàng (đã bao gồm thuế GTGT 8%)</t>
         </is>
       </c>
-      <c r="B22" s="28" t="n"/>
-      <c r="C22" s="28" t="n"/>
-      <c r="D22" s="28" t="n"/>
-      <c r="E22" s="28" t="n"/>
-      <c r="F22" s="29">
-        <f>SUM(F20:F21)</f>
+      <c r="B23" s="28" t="n"/>
+      <c r="C23" s="28" t="n"/>
+      <c r="D23" s="28" t="n"/>
+      <c r="E23" s="28" t="n"/>
+      <c r="F23" s="29">
+        <f>SUM(F20:F22)</f>
         <v/>
       </c>
-      <c r="G22" s="30" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="31" t="inlineStr">
+      <c r="G23" s="30" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t>TỔNG CỘNG THANH TOÁN</t>
         </is>
       </c>
-      <c r="B23" s="31" t="n"/>
-      <c r="C23" s="31" t="n"/>
-      <c r="D23" s="31" t="n"/>
-      <c r="E23" s="31" t="n"/>
-      <c r="F23" s="32">
-        <f>F22</f>
+      <c r="B24" s="31" t="n"/>
+      <c r="C24" s="31" t="n"/>
+      <c r="D24" s="31" t="n"/>
+      <c r="E24" s="31" t="n"/>
+      <c r="F24" s="32">
+        <f>F23</f>
         <v/>
       </c>
-      <c r="G23" s="33" t="n"/>
-    </row>
-    <row r="24" ht="22" customHeight="1">
-      <c r="A24" s="34" t="inlineStr">
+      <c r="G24" s="33" t="n"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="34" t="inlineStr">
         <is>
           <t>Bằng chữ: Bốn mươi lăm triệu không trăm mười chín nghìn bốn trăm đồng.</t>
         </is>
       </c>
-      <c r="B24" s="34" t="n"/>
-      <c r="C24" s="34" t="n"/>
-      <c r="D24" s="34" t="n"/>
-      <c r="E24" s="34" t="n"/>
-      <c r="F24" s="34" t="n"/>
-      <c r="G24" s="34" t="n"/>
-    </row>
-    <row r="25" ht="12" customHeight="1"/>
-    <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="35" t="inlineStr">
+      <c r="B25" s="34" t="n"/>
+      <c r="C25" s="34" t="n"/>
+      <c r="D25" s="34" t="n"/>
+      <c r="E25" s="34" t="n"/>
+      <c r="F25" s="34" t="n"/>
+      <c r="G25" s="34" t="n"/>
+    </row>
+    <row r="26" ht="12" customHeight="1"/>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="35" t="inlineStr">
         <is>
           <t>ĐIỀU KHOẢN THƯƠNG MẠI</t>
         </is>
       </c>
-      <c r="B26" s="35" t="n"/>
-      <c r="C26" s="35" t="n"/>
-      <c r="D26" s="35" t="n"/>
-      <c r="E26" s="35" t="n"/>
-      <c r="F26" s="35" t="n"/>
-      <c r="G26" s="35" t="n"/>
-    </row>
-    <row r="27" ht="17.5" customHeight="1">
-      <c r="A27" s="36" t="inlineStr">
-        <is>
-          <t>1. Đơn giá trên đã bao gồm thuế GTGT 8%.</t>
-        </is>
-      </c>
-      <c r="B27" s="36" t="n"/>
-      <c r="C27" s="36" t="n"/>
-      <c r="D27" s="36" t="n"/>
-      <c r="E27" s="36" t="n"/>
-      <c r="F27" s="36" t="n"/>
-      <c r="G27" s="36" t="n"/>
+      <c r="B27" s="35" t="n"/>
+      <c r="C27" s="35" t="n"/>
+      <c r="D27" s="35" t="n"/>
+      <c r="E27" s="35" t="n"/>
+      <c r="F27" s="35" t="n"/>
+      <c r="G27" s="35" t="n"/>
     </row>
     <row r="28" ht="17.5" customHeight="1">
       <c r="A28" s="36" t="inlineStr">
         <is>
-          <t>2. Hiệu lực báo giá: 30 ngày kể từ ngày báo giá.</t>
+          <t>1. Đơn giá trên đã bao gồm thuế GTGT 8%.</t>
         </is>
       </c>
       <c r="B28" s="36" t="n"/>
@@ -1239,7 +1254,7 @@
     <row r="29" ht="17.5" customHeight="1">
       <c r="A29" s="36" t="inlineStr">
         <is>
-          <t>3. Thời gian giao hàng: trong vòng 03 ngày kể từ khi Quý khách xác nhận đặt hàng.</t>
+          <t>2. Hiệu lực báo giá: 30 ngày kể từ ngày báo giá.</t>
         </is>
       </c>
       <c r="B29" s="36" t="n"/>
@@ -1252,7 +1267,7 @@
     <row r="30" ht="17.5" customHeight="1">
       <c r="A30" s="36" t="inlineStr">
         <is>
-          <t>4. Địa điểm giao hàng: tại kho của Quý khách.</t>
+          <t>3. Thời gian giao hàng: trong vòng 03 ngày kể từ khi Quý khách xác nhận đặt hàng.</t>
         </is>
       </c>
       <c r="B30" s="36" t="n"/>
@@ -1265,7 +1280,7 @@
     <row r="31" ht="17.5" customHeight="1">
       <c r="A31" s="36" t="inlineStr">
         <is>
-          <t>5. Thanh toán: chuyển khoản, 100% khi nhận hàng.</t>
+          <t>4. Địa điểm giao hàng: tại kho của Quý khách.</t>
         </is>
       </c>
       <c r="B31" s="36" t="n"/>
@@ -1275,10 +1290,10 @@
       <c r="F31" s="36" t="n"/>
       <c r="G31" s="36" t="n"/>
     </row>
-    <row r="32" ht="30" customHeight="1">
+    <row r="32" ht="17.5" customHeight="1">
       <c r="A32" s="36" t="inlineStr">
         <is>
-          <t>6. Thông tin chuyển khoản: Số TK 1066217478 – Ngân hàng TMCP Ngoại thương Việt Nam (Vietcombank) – Chủ tài khoản: CT TNHH KY THUAT CONG TRINH BLT.</t>
+          <t>5. Thanh toán: chuyển khoản, 100% khi nhận hàng.</t>
         </is>
       </c>
       <c r="B32" s="36" t="n"/>
@@ -1288,65 +1303,78 @@
       <c r="F32" s="36" t="n"/>
       <c r="G32" s="36" t="n"/>
     </row>
-    <row r="33" ht="6" customHeight="1"/>
-    <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="16" t="inlineStr">
+    <row r="33" ht="30" customHeight="1">
+      <c r="A33" s="36" t="inlineStr">
+        <is>
+          <t>6. Thông tin chuyển khoản: Số TK 1066217478 – Ngân hàng TMCP Ngoại thương Việt Nam (Vietcombank) – Chủ tài khoản: CT TNHH KY THUAT CONG TRINH BLT.</t>
+        </is>
+      </c>
+      <c r="B33" s="36" t="n"/>
+      <c r="C33" s="36" t="n"/>
+      <c r="D33" s="36" t="n"/>
+      <c r="E33" s="36" t="n"/>
+      <c r="F33" s="36" t="n"/>
+      <c r="G33" s="36" t="n"/>
+    </row>
+    <row r="34" ht="6" customHeight="1"/>
+    <row r="35" ht="18" customHeight="1">
+      <c r="A35" s="16" t="inlineStr">
         <is>
           <t>Rất mong nhận được sự hợp tác của Quý khách. Trân trọng!</t>
         </is>
       </c>
-      <c r="B34" s="16" t="n"/>
-      <c r="C34" s="16" t="n"/>
-      <c r="D34" s="16" t="n"/>
-      <c r="E34" s="16" t="n"/>
-      <c r="F34" s="16" t="n"/>
-      <c r="G34" s="16" t="n"/>
-    </row>
-    <row r="35" ht="12" customHeight="1"/>
-    <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="37" t="inlineStr">
+      <c r="B35" s="16" t="n"/>
+      <c r="C35" s="16" t="n"/>
+      <c r="D35" s="16" t="n"/>
+      <c r="E35" s="16" t="n"/>
+      <c r="F35" s="16" t="n"/>
+      <c r="G35" s="16" t="n"/>
+    </row>
+    <row r="36" ht="12" customHeight="1"/>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="37" t="inlineStr">
         <is>
           <t>XÁC NHẬN CỦA KHÁCH HÀNG</t>
         </is>
       </c>
-      <c r="B36" s="37" t="n"/>
-      <c r="C36" s="37" t="n"/>
-      <c r="E36" s="37" t="inlineStr">
+      <c r="B37" s="37" t="n"/>
+      <c r="C37" s="37" t="n"/>
+      <c r="E37" s="37" t="inlineStr">
         <is>
           <t>GIÁM ĐỐC</t>
         </is>
       </c>
-      <c r="F36" s="37" t="n"/>
-      <c r="G36" s="37" t="n"/>
-    </row>
-    <row r="37" ht="15" customHeight="1">
-      <c r="A37" s="38" t="inlineStr">
+      <c r="F37" s="37" t="n"/>
+      <c r="G37" s="37" t="n"/>
+    </row>
+    <row r="38" ht="15" customHeight="1">
+      <c r="A38" s="38" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ tên)</t>
         </is>
       </c>
-      <c r="B37" s="38" t="n"/>
-      <c r="C37" s="38" t="n"/>
-      <c r="E37" s="38" t="inlineStr">
+      <c r="B38" s="38" t="n"/>
+      <c r="C38" s="38" t="n"/>
+      <c r="E38" s="38" t="inlineStr">
         <is>
           <t>(Ký, đóng dấu, ghi rõ họ tên)</t>
         </is>
       </c>
-      <c r="F37" s="38" t="n"/>
-      <c r="G37" s="38" t="n"/>
-    </row>
-    <row r="38" ht="16" customHeight="1"/>
+      <c r="F38" s="38" t="n"/>
+      <c r="G38" s="38" t="n"/>
+    </row>
     <row r="39" ht="16" customHeight="1"/>
     <row r="40" ht="16" customHeight="1"/>
     <row r="41" ht="16" customHeight="1"/>
-    <row r="42" ht="20" customHeight="1">
-      <c r="E42" s="39" t="inlineStr">
+    <row r="42" ht="16" customHeight="1"/>
+    <row r="43" ht="20" customHeight="1">
+      <c r="E43" s="39" t="inlineStr">
         <is>
           <t>HỒ VĂN BÌNH</t>
         </is>
       </c>
-      <c r="F42" s="39" t="n"/>
-      <c r="G42" s="39" t="n"/>
+      <c r="F43" s="39" t="n"/>
+      <c r="G43" s="39" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="33">
@@ -1354,35 +1382,35 @@
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E13:G13"/>
     <mergeCell ref="A17:G17"/>
+    <mergeCell ref="A24:E24"/>
     <mergeCell ref="A8:G8"/>
     <mergeCell ref="A37:C37"/>
+    <mergeCell ref="A35:G35"/>
     <mergeCell ref="B1:G1"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A12:C12"/>
     <mergeCell ref="E15:G15"/>
     <mergeCell ref="A28:G28"/>
-    <mergeCell ref="E36:G36"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="E11:G11"/>
     <mergeCell ref="A31:G31"/>
     <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A34:G34"/>
-    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A38:C38"/>
     <mergeCell ref="A13:C13"/>
     <mergeCell ref="E37:G37"/>
     <mergeCell ref="B4:G4"/>
     <mergeCell ref="E12:G12"/>
     <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A25:G25"/>
     <mergeCell ref="A15:C15"/>
-    <mergeCell ref="A22:E22"/>
+    <mergeCell ref="E43:G43"/>
     <mergeCell ref="B3:G3"/>
-    <mergeCell ref="E42:G42"/>
-    <mergeCell ref="A36:C36"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="E14:G14"/>
     <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="E38:G38"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.45" bottom="0.6" header="0.5" footer="0.25"/>

</xml_diff>

<commit_message>
Báo giá BG-2026/002: số lượng dây 1x4 là 20.000 m
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
+++ b/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
@@ -1139,7 +1139,9 @@
           <t>m</t>
         </is>
       </c>
-      <c r="D21" s="25" t="n"/>
+      <c r="D21" s="25" t="n">
+        <v>20000</v>
+      </c>
       <c r="E21" s="25" t="n">
         <v>18000</v>
       </c>
@@ -1147,11 +1149,7 @@
         <f>IF(OR(D21="",E21=""),"",ROUND(D21*E21,0))</f>
         <v/>
       </c>
-      <c r="G21" s="27" t="inlineStr">
-        <is>
-          <t>Chờ số lượng</t>
-        </is>
-      </c>
+      <c r="G21" s="27" t="inlineStr"/>
     </row>
     <row r="22" ht="19" customHeight="1">
       <c r="A22" s="18" t="n">
@@ -1214,7 +1212,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>Bằng chữ: Bốn mươi lăm triệu không trăm mười chín nghìn bốn trăm đồng.</t>
+          <t>Bằng chữ: Bốn trăm lẻ năm triệu không trăm mười chín nghìn bốn trăm đồng.</t>
         </is>
       </c>
       <c r="B25" s="34" t="n"/>

</xml_diff>

<commit_message>
Báo giá BG-2026/002: đơn giá dây ô van 2x2.5 là 25.000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
+++ b/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
@@ -1169,7 +1169,7 @@
         <v>1400</v>
       </c>
       <c r="E22" s="20" t="n">
-        <v>24096</v>
+        <v>25000</v>
       </c>
       <c r="F22" s="21">
         <f>IF(OR(D22="",E22=""),"",ROUND(D22*E22,0))</f>
@@ -1212,7 +1212,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>Bằng chữ: Bốn trăm lẻ năm triệu không trăm mười chín nghìn bốn trăm đồng.</t>
+          <t>Bằng chữ: Bốn trăm lẻ sáu triệu hai trăm tám mươi lăm nghìn đồng chẵn.</t>
         </is>
       </c>
       <c r="B25" s="34" t="n"/>

</xml_diff>

<commit_message>
Báo giá BG-2026/002: đơn giá dây mềm 1x2.5 là 15.000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
+++ b/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
@@ -1117,7 +1117,7 @@
         <v>1000</v>
       </c>
       <c r="E20" s="20" t="n">
-        <v>11285</v>
+        <v>15000</v>
       </c>
       <c r="F20" s="21">
         <f>IF(OR(D20="",E20=""),"",ROUND(D20*E20,0))</f>
@@ -1212,7 +1212,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>Bằng chữ: Bốn trăm lẻ sáu triệu hai trăm tám mươi lăm nghìn đồng chẵn.</t>
+          <t>Bằng chữ: Bốn trăm mười triệu đồng chẵn.</t>
         </is>
       </c>
       <c r="B25" s="34" t="n"/>

</xml_diff>

<commit_message>
Báo giá BG-2026/002: đơn giá dây 1x4 là 20.000
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
+++ b/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
@@ -1143,7 +1143,7 @@
         <v>20000</v>
       </c>
       <c r="E21" s="25" t="n">
-        <v>18000</v>
+        <v>20000</v>
       </c>
       <c r="F21" s="26">
         <f>IF(OR(D21="",E21=""),"",ROUND(D21*E21,0))</f>
@@ -1212,7 +1212,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>Bằng chữ: Bốn trăm mười triệu đồng chẵn.</t>
+          <t>Bằng chữ: Bốn trăm năm mươi triệu đồng chẵn.</t>
         </is>
       </c>
       <c r="B25" s="34" t="n"/>

</xml_diff>

<commit_message>
Báo giá BG-2026/002: cập nhật số lượng 200 m, 340 m, 100 m
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
+++ b/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="D20" s="20" t="n">
-        <v>1000</v>
+        <v>200</v>
       </c>
       <c r="E20" s="20" t="n">
         <v>15000</v>
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="D21" s="25" t="n">
-        <v>20000</v>
+        <v>340</v>
       </c>
       <c r="E21" s="25" t="n">
         <v>20000</v>
@@ -1166,7 +1166,7 @@
         </is>
       </c>
       <c r="D22" s="20" t="n">
-        <v>1400</v>
+        <v>100</v>
       </c>
       <c r="E22" s="20" t="n">
         <v>25000</v>
@@ -1212,7 +1212,7 @@
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>Bằng chữ: Bốn trăm năm mươi triệu đồng chẵn.</t>
+          <t>Bằng chữ: Mười hai triệu ba trăm nghìn đồng chẵn.</t>
         </is>
       </c>
       <c r="B25" s="34" t="n"/>

</xml_diff>

<commit_message>
lap-bao-gia: thêm kiểu mẫu thi công truyền thống, báo giá D20 theo mẫu mới
- Kiểu xay-dung (Times New Roman, đen trắng) theo mẫu BẢNG BÁO GIÁ thi công:
  logo + số BG trái, công ty phải, Kính gửi, câu mở đầu có công trình và địa
  điểm, bảng Nội dung công việc / Khối lượng (tạm tính), Ghi chú, liên hệ,
  ngày lập + chữ ký; hỗ trợ song ngữ Việt – Trung
- Kiểu hiện đại: đầu trang logo + tên công ty trái, tiêu đề + số/ngày/hiệu lực
  phải; khung Bên báo giá / Kính gửi khách hàng; giá gồm VAT chỉ một dòng tổng;
  số lượng, đơn giá chữ xanh; tên dài tự thu nhỏ
- Hồ sơ BLT: tên/địa chỉ tiếng Trung, tên viết thường, nơi lập, kiểu mặc định
- Không lặp tiêu đề bảng khi bảng nằm gọn trang 1; mẫu trống gọn 1 trang
- Xuất lại báo giá D20 (Việt, song ngữ), mẫu BLT (thi công, hiện đại)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EWvKCUnFhSdC1AiEF1AweY
</commit_message>
<xml_diff>
--- a/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
+++ b/bao-gia/BLT/Day-dien/Bao-gia-BLT-Day-dien-BG-2026-002.xlsx
@@ -10,8 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Báo giá" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Báo giá'!$19:$19</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'Báo giá'!$A$1:$G$43</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Báo giá'!$17:$17</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'Báo giá'!$A$1:$G$40</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -32,7 +32,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="000D2B66"/>
-      <sz val="16"/>
+      <sz val="12"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -43,7 +43,7 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="000D2B66"/>
-      <sz val="22"/>
+      <sz val="20"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -69,6 +69,11 @@
     </font>
     <font>
       <name val="Arial"/>
+      <color rgb="001F4FBF"/>
+      <sz val="9.5"/>
+    </font>
+    <font>
+      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00000000"/>
       <sz val="9.5"/>
@@ -77,12 +82,6 @@
       <name val="Arial"/>
       <color rgb="00404040"/>
       <sz val="8.5"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00000000"/>
-      <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -149,7 +148,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="14">
     <border>
       <left/>
       <right/>
@@ -242,31 +241,29 @@
         <color rgb="00C9D1DC"/>
       </bottom>
     </border>
-    <border>
-      <top style="medium">
-        <color rgb="000D2B66"/>
-      </top>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="bottom" indent="6"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="6"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
@@ -306,13 +303,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="8" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -321,22 +318,13 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="7" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="3" fontId="8" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="9" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="3" fontId="10" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -449,9 +437,9 @@
       <col>0</col>
       <colOff>19050</colOff>
       <row>0</row>
-      <rowOff>28575</rowOff>
+      <rowOff>133350</rowOff>
     </from>
-    <ext cx="876300" cy="876300"/>
+    <ext cx="800100" cy="800100"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -761,19 +749,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5.5" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="38.5" customWidth="1" min="2" max="2"/>
+    <col width="9.5" customWidth="1" min="3" max="3"/>
     <col width="9" customWidth="1" min="4" max="4"/>
     <col width="14.5" customWidth="1" min="5" max="5"/>
     <col width="16.5" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1" ht="30" customHeight="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
           <t>CÔNG TY TNHH KỸ THUẬT CÔNG TRÌNH BLT</t>
@@ -781,110 +769,39 @@
       </c>
       <c r="C1" s="1" t="n"/>
       <c r="D1" s="1" t="n"/>
-      <c r="E1" s="1" t="n"/>
-      <c r="F1" s="1" t="n"/>
-      <c r="G1" s="1" t="n"/>
-    </row>
-    <row r="2" ht="15" customHeight="1">
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Địa chỉ: Số 2A đường Nguyễn Khánh Toàn, khối Trường Phúc, phường Trường Vinh, tỉnh Nghệ An, Việt Nam</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>BẢNG BÁO GIÁ</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="17" customHeight="1">
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>MST: 2902269718</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n"/>
+      <c r="D2" s="3" t="n"/>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>QUOTATION</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="n"/>
+      <c r="G2" s="4" t="n"/>
     </row>
     <row r="3" ht="15" customHeight="1">
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>MST: 2902269718   |   Điện thoại: 0984 586 089</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-    </row>
-    <row r="4" ht="15" customHeight="1">
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>Email: hobinh150589@gmail.com</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-    </row>
-    <row r="5" ht="10" customHeight="1">
-      <c r="A5" s="3" t="n"/>
-      <c r="B5" s="3" t="n"/>
-      <c r="C5" s="3" t="n"/>
-      <c r="D5" s="3" t="n"/>
-      <c r="E5" s="3" t="n"/>
-      <c r="F5" s="3" t="n"/>
-      <c r="G5" s="3" t="n"/>
-    </row>
-    <row r="6" ht="4" customHeight="1">
-      <c r="A6" s="4" t="n"/>
-      <c r="B6" s="4" t="n"/>
-      <c r="C6" s="4" t="n"/>
-      <c r="D6" s="4" t="n"/>
-      <c r="E6" s="4" t="n"/>
-      <c r="F6" s="4" t="n"/>
-      <c r="G6" s="4" t="n"/>
-    </row>
-    <row r="7" ht="10" customHeight="1"/>
-    <row r="8" ht="34" customHeight="1">
-      <c r="A8" s="5" t="inlineStr">
-        <is>
-          <t>BẢNG BÁO GIÁ</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="n"/>
-      <c r="C8" s="5" t="n"/>
-      <c r="D8" s="5" t="n"/>
-      <c r="E8" s="5" t="n"/>
-      <c r="F8" s="5" t="n"/>
-      <c r="G8" s="5" t="n"/>
-    </row>
-    <row r="9" ht="16" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>QUOTATION</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="n"/>
-      <c r="C9" s="6" t="n"/>
-      <c r="D9" s="6" t="n"/>
-      <c r="E9" s="6" t="n"/>
-      <c r="F9" s="6" t="n"/>
-      <c r="G9" s="6" t="n"/>
-    </row>
-    <row r="10" ht="10" customHeight="1"/>
-    <row r="11" ht="20" customHeight="1">
-      <c r="A11" s="7" t="inlineStr">
-        <is>
-          <t>THÔNG TIN KHÁCH HÀNG</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="9" t="n"/>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>THÔNG TIN BÁO GIÁ</t>
-        </is>
-      </c>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="9" t="n"/>
-    </row>
-    <row r="12" ht="17.5" customHeight="1">
-      <c r="A12" s="10" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Điện thoại: 0984 586 089</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -892,7 +809,7 @@
               <color rgb="00595959"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Kính gửi: </t>
+            <t xml:space="preserve">Số báo giá: </t>
           </r>
           <r>
             <rPr>
@@ -901,13 +818,22 @@
               <color rgb="00000000"/>
               <sz val="9.5"/>
             </rPr>
-            <t>Quý khách hàng</t>
-          </r>
-        </is>
-      </c>
-      <c r="B12" s="11" t="n"/>
-      <c r="C12" s="12" t="n"/>
-      <c r="E12" s="10" t="inlineStr">
+            <t>BG-2026/002</t>
+          </r>
+        </is>
+      </c>
+      <c r="F3" s="5" t="n"/>
+      <c r="G3" s="5" t="n"/>
+    </row>
+    <row r="4" ht="15" customHeight="1">
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Email: hobinh150589@gmail.com</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -915,7 +841,112 @@
               <color rgb="00595959"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Số báo giá: </t>
+            <t xml:space="preserve">Ngày báo giá: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t>12/10/2026</t>
+          </r>
+        </is>
+      </c>
+      <c r="F4" s="5" t="n"/>
+      <c r="G4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="15" customHeight="1">
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00595959"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t xml:space="preserve">Hiệu lực: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t>30 ngày</t>
+          </r>
+        </is>
+      </c>
+      <c r="F5" s="5" t="n"/>
+      <c r="G5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="10" customHeight="1">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+      <c r="F6" s="6" t="n"/>
+      <c r="G6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="4" customHeight="1">
+      <c r="A7" s="7" t="n"/>
+      <c r="B7" s="7" t="n"/>
+      <c r="C7" s="7" t="n"/>
+      <c r="D7" s="7" t="n"/>
+      <c r="E7" s="7" t="n"/>
+      <c r="F7" s="7" t="n"/>
+      <c r="G7" s="7" t="n"/>
+    </row>
+    <row r="8" ht="10" customHeight="1"/>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>BÊN BÁO GIÁ</t>
+        </is>
+      </c>
+      <c r="B9" s="9" t="n"/>
+      <c r="C9" s="10" t="n"/>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>KÍNH GỬI KHÁCH HÀNG</t>
+        </is>
+      </c>
+      <c r="F9" s="9" t="n"/>
+      <c r="G9" s="10" t="n"/>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00595959"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t xml:space="preserve">Địa chỉ: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t>Số 2A đường Nguyễn Khánh Toàn, khối Trường Phúc, phường Trường Vinh, tỉnh Nghệ An, Việt Nam</t>
+          </r>
+        </is>
+      </c>
+      <c r="B10" s="12" t="n"/>
+      <c r="C10" s="13" t="n"/>
+      <c r="E10" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00595959"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t xml:space="preserve">Kính gửi: </t>
           </r>
           <r>
             <rPr>
@@ -924,15 +955,94 @@
               <color rgb="00000000"/>
               <sz val="9.5"/>
             </rPr>
-            <t>BG-2026/002</t>
-          </r>
-        </is>
-      </c>
-      <c r="F12" s="11" t="n"/>
-      <c r="G12" s="12" t="n"/>
+            <t>Quý khách hàng</t>
+          </r>
+        </is>
+      </c>
+      <c r="F10" s="12" t="n"/>
+      <c r="G10" s="13" t="n"/>
+    </row>
+    <row r="11" ht="17.5" customHeight="1">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00595959"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t xml:space="preserve">Người phụ trách: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t>HỒ VĂN BÌNH – Giám đốc</t>
+          </r>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n"/>
+      <c r="C11" s="13" t="n"/>
+      <c r="E11" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00595959"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t xml:space="preserve">Người liên hệ: </t>
+          </r>
+        </is>
+      </c>
+      <c r="F11" s="12" t="n"/>
+      <c r="G11" s="13" t="n"/>
+    </row>
+    <row r="12" ht="17.5" customHeight="1">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00595959"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t xml:space="preserve">Số tài khoản: </t>
+          </r>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00000000"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t>1066217478 – Vietcombank</t>
+          </r>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n"/>
+      <c r="C12" s="13" t="n"/>
+      <c r="E12" s="11" t="inlineStr">
+        <is>
+          <r>
+            <rPr>
+              <rFont val="Arial"/>
+              <color rgb="00595959"/>
+              <sz val="9.5"/>
+            </rPr>
+            <t xml:space="preserve">Điện thoại: </t>
+          </r>
+        </is>
+      </c>
+      <c r="F12" s="12" t="n"/>
+      <c r="G12" s="13" t="n"/>
     </row>
     <row r="13" ht="17.5" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+      <c r="A13" s="14" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="16" t="n"/>
+      <c r="E13" s="14" t="inlineStr">
         <is>
           <r>
             <rPr>
@@ -940,279 +1050,192 @@
               <color rgb="00595959"/>
               <sz val="9.5"/>
             </rPr>
-            <t xml:space="preserve">Người liên hệ: </t>
-          </r>
-        </is>
-      </c>
-      <c r="B13" s="11" t="n"/>
-      <c r="C13" s="12" t="n"/>
-      <c r="E13" s="10" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00595959"/>
-              <sz val="9.5"/>
-            </rPr>
-            <t xml:space="preserve">Ngày báo giá: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="9.5"/>
-            </rPr>
-            <t>12/10/2026</t>
-          </r>
-        </is>
-      </c>
-      <c r="F13" s="11" t="n"/>
-      <c r="G13" s="12" t="n"/>
-    </row>
-    <row r="14" ht="17.5" customHeight="1">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00595959"/>
-              <sz val="9.5"/>
-            </rPr>
-            <t xml:space="preserve">Điện thoại: </t>
-          </r>
-        </is>
-      </c>
-      <c r="B14" s="11" t="n"/>
-      <c r="C14" s="12" t="n"/>
-      <c r="E14" s="10" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00595959"/>
-              <sz val="9.5"/>
-            </rPr>
-            <t xml:space="preserve">Hiệu lực: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="9.5"/>
-            </rPr>
-            <t>30 ngày</t>
-          </r>
-        </is>
-      </c>
-      <c r="F14" s="11" t="n"/>
-      <c r="G14" s="12" t="n"/>
-    </row>
-    <row r="15" ht="17.5" customHeight="1">
-      <c r="A15" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00595959"/>
-              <sz val="9.5"/>
-            </rPr>
             <t xml:space="preserve">Địa chỉ: </t>
           </r>
         </is>
       </c>
-      <c r="B15" s="14" t="n"/>
-      <c r="C15" s="15" t="n"/>
-      <c r="E15" s="13" t="inlineStr">
-        <is>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00595959"/>
-              <sz val="9.5"/>
-            </rPr>
-            <t xml:space="preserve">Người phụ trách: </t>
-          </r>
-          <r>
-            <rPr>
-              <rFont val="Arial"/>
-              <color rgb="00000000"/>
-              <sz val="9.5"/>
-            </rPr>
-            <t>HỒ VĂN BÌNH – 0984 586 089</t>
-          </r>
-        </is>
-      </c>
-      <c r="F15" s="14" t="n"/>
-      <c r="G15" s="15" t="n"/>
-    </row>
-    <row r="16" ht="10" customHeight="1"/>
-    <row r="17" ht="31" customHeight="1">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="F13" s="15" t="n"/>
+      <c r="G13" s="16" t="n"/>
+    </row>
+    <row r="14" ht="10" customHeight="1"/>
+    <row r="15" ht="31" customHeight="1">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>CÔNG TY TNHH KỸ THUẬT CÔNG TRÌNH BLT trân trọng cảm ơn Quý khách đã quan tâm đến sản phẩm, dịch vụ của chúng tôi. Chúng tôi xin gửi tới Quý khách bảng báo giá như sau:</t>
         </is>
       </c>
-      <c r="B17" s="16" t="n"/>
-      <c r="C17" s="16" t="n"/>
-      <c r="D17" s="16" t="n"/>
-      <c r="E17" s="16" t="n"/>
-      <c r="F17" s="16" t="n"/>
-      <c r="G17" s="16" t="n"/>
-    </row>
-    <row r="18" ht="8" customHeight="1"/>
-    <row r="19" ht="32" customHeight="1">
-      <c r="A19" s="17" t="inlineStr">
+      <c r="B15" s="17" t="n"/>
+      <c r="C15" s="17" t="n"/>
+      <c r="D15" s="17" t="n"/>
+      <c r="E15" s="17" t="n"/>
+      <c r="F15" s="17" t="n"/>
+      <c r="G15" s="17" t="n"/>
+    </row>
+    <row r="16" ht="8" customHeight="1"/>
+    <row r="17" ht="32" customHeight="1">
+      <c r="A17" s="18" t="inlineStr">
         <is>
           <t>STT</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B17" s="18" t="inlineStr">
         <is>
           <t>Tên hàng hóa / Quy cách kỹ thuật</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C17" s="18" t="inlineStr">
         <is>
           <t>ĐVT</t>
         </is>
       </c>
-      <c r="D19" s="17" t="inlineStr">
+      <c r="D17" s="18" t="inlineStr">
         <is>
           <t>Số lượng</t>
         </is>
       </c>
-      <c r="E19" s="17" t="inlineStr">
+      <c r="E17" s="18" t="inlineStr">
         <is>
           <t>Đơn giá
 (VNĐ)</t>
         </is>
       </c>
-      <c r="F19" s="17" t="inlineStr">
+      <c r="F17" s="18" t="inlineStr">
         <is>
           <t>Thành tiền
 (VNĐ)</t>
         </is>
       </c>
-      <c r="G19" s="17" t="inlineStr">
+      <c r="G17" s="18" t="inlineStr">
         <is>
           <t>Ghi chú</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="19" customHeight="1">
-      <c r="A20" s="18" t="n">
+    <row r="18" ht="19" customHeight="1">
+      <c r="A18" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="B20" s="19" t="inlineStr">
+      <c r="B18" s="20" t="inlineStr">
         <is>
           <t>Dây điện mềm Cu/PVC 1×2.5mm² – 450/750V</t>
         </is>
       </c>
-      <c r="C20" s="18" t="inlineStr">
+      <c r="C18" s="19" t="inlineStr">
         <is>
           <t>m</t>
         </is>
       </c>
-      <c r="D20" s="20" t="n">
+      <c r="D18" s="21" t="n">
         <v>200</v>
       </c>
-      <c r="E20" s="20" t="n">
+      <c r="E18" s="21" t="n">
         <v>15000</v>
       </c>
-      <c r="F20" s="21">
+      <c r="F18" s="22">
+        <f>IF(OR(D18="",E18=""),"",ROUND(D18*E18,0))</f>
+        <v/>
+      </c>
+      <c r="G18" s="23" t="inlineStr"/>
+    </row>
+    <row r="19" ht="19" customHeight="1">
+      <c r="A19" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="B19" s="25" t="inlineStr">
+        <is>
+          <t>Dây điện IS 1×4</t>
+        </is>
+      </c>
+      <c r="C19" s="24" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D19" s="26" t="n">
+        <v>340</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <v>20000</v>
+      </c>
+      <c r="F19" s="27">
+        <f>IF(OR(D19="",E19=""),"",ROUND(D19*E19,0))</f>
+        <v/>
+      </c>
+      <c r="G19" s="28" t="inlineStr"/>
+    </row>
+    <row r="20" ht="30" customHeight="1">
+      <c r="A20" s="19" t="n">
+        <v>3</v>
+      </c>
+      <c r="B20" s="20" t="inlineStr">
+        <is>
+          <t>Dây điện ô van Cu/PVC/PVC 2×2.5mm² – 300/500V</t>
+        </is>
+      </c>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="D20" s="21" t="n">
+        <v>100</v>
+      </c>
+      <c r="E20" s="21" t="n">
+        <v>25000</v>
+      </c>
+      <c r="F20" s="22">
         <f>IF(OR(D20="",E20=""),"",ROUND(D20*E20,0))</f>
         <v/>
       </c>
-      <c r="G20" s="22" t="inlineStr"/>
-    </row>
-    <row r="21" ht="19" customHeight="1">
-      <c r="A21" s="23" t="n">
-        <v>2</v>
-      </c>
-      <c r="B21" s="24" t="inlineStr">
-        <is>
-          <t>Dây điện IS 1×4</t>
-        </is>
-      </c>
-      <c r="C21" s="23" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D21" s="25" t="n">
-        <v>340</v>
-      </c>
-      <c r="E21" s="25" t="n">
-        <v>20000</v>
-      </c>
-      <c r="F21" s="26">
-        <f>IF(OR(D21="",E21=""),"",ROUND(D21*E21,0))</f>
+      <c r="G20" s="23" t="inlineStr"/>
+    </row>
+    <row r="21" ht="24" customHeight="1">
+      <c r="A21" s="29" t="inlineStr">
+        <is>
+          <t>TỔNG CỘNG THANH TOÁN (đã gồm VAT 8%)</t>
+        </is>
+      </c>
+      <c r="B21" s="29" t="n"/>
+      <c r="C21" s="29" t="n"/>
+      <c r="D21" s="29" t="n"/>
+      <c r="E21" s="29" t="n"/>
+      <c r="F21" s="30">
+        <f>SUM(F18:F20)</f>
         <v/>
       </c>
-      <c r="G21" s="27" t="inlineStr"/>
-    </row>
-    <row r="22" ht="19" customHeight="1">
-      <c r="A22" s="18" t="n">
-        <v>3</v>
-      </c>
-      <c r="B22" s="19" t="inlineStr">
-        <is>
-          <t>Dây điện ô van Cu/PVC/PVC 2×2.5mm² – 300/500V</t>
-        </is>
-      </c>
-      <c r="C22" s="18" t="inlineStr">
-        <is>
-          <t>m</t>
-        </is>
-      </c>
-      <c r="D22" s="20" t="n">
-        <v>100</v>
-      </c>
-      <c r="E22" s="20" t="n">
-        <v>25000</v>
-      </c>
-      <c r="F22" s="21">
-        <f>IF(OR(D22="",E22=""),"",ROUND(D22*E22,0))</f>
-        <v/>
-      </c>
-      <c r="G22" s="22" t="inlineStr"/>
-    </row>
-    <row r="23" ht="20" customHeight="1">
-      <c r="A23" s="28" t="inlineStr">
-        <is>
-          <t>Cộng tiền hàng (đã bao gồm thuế GTGT 8%)</t>
-        </is>
-      </c>
-      <c r="B23" s="28" t="n"/>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="28" t="n"/>
-      <c r="E23" s="28" t="n"/>
-      <c r="F23" s="29">
-        <f>SUM(F20:F22)</f>
-        <v/>
-      </c>
-      <c r="G23" s="30" t="n"/>
-    </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="31" t="inlineStr">
-        <is>
-          <t>TỔNG CỘNG THANH TOÁN</t>
-        </is>
-      </c>
-      <c r="B24" s="31" t="n"/>
-      <c r="C24" s="31" t="n"/>
-      <c r="D24" s="31" t="n"/>
-      <c r="E24" s="31" t="n"/>
-      <c r="F24" s="32">
-        <f>F23</f>
-        <v/>
-      </c>
+      <c r="G21" s="31" t="n"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>Bằng chữ: Mười hai triệu ba trăm nghìn đồng chẵn.</t>
+        </is>
+      </c>
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="32" t="n"/>
+      <c r="F22" s="32" t="n"/>
+      <c r="G22" s="32" t="n"/>
+    </row>
+    <row r="23" ht="12" customHeight="1"/>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="33" t="inlineStr">
+        <is>
+          <t>ĐIỀU KHOẢN THƯƠNG MẠI</t>
+        </is>
+      </c>
+      <c r="B24" s="33" t="n"/>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="33" t="n"/>
+      <c r="E24" s="33" t="n"/>
+      <c r="F24" s="33" t="n"/>
       <c r="G24" s="33" t="n"/>
     </row>
-    <row r="25" ht="22" customHeight="1">
+    <row r="25" ht="17.5" customHeight="1">
       <c r="A25" s="34" t="inlineStr">
         <is>
-          <t>Bằng chữ: Mười hai triệu ba trăm nghìn đồng chẵn.</t>
+          <t>1. Đơn giá trên đã bao gồm thuế GTGT 8%.</t>
         </is>
       </c>
       <c r="B25" s="34" t="n"/>
@@ -1222,193 +1245,168 @@
       <c r="F25" s="34" t="n"/>
       <c r="G25" s="34" t="n"/>
     </row>
-    <row r="26" ht="12" customHeight="1"/>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="35" t="inlineStr">
-        <is>
-          <t>ĐIỀU KHOẢN THƯƠNG MẠI</t>
-        </is>
-      </c>
-      <c r="B27" s="35" t="n"/>
-      <c r="C27" s="35" t="n"/>
-      <c r="D27" s="35" t="n"/>
-      <c r="E27" s="35" t="n"/>
-      <c r="F27" s="35" t="n"/>
-      <c r="G27" s="35" t="n"/>
+    <row r="26" ht="17.5" customHeight="1">
+      <c r="A26" s="34" t="inlineStr">
+        <is>
+          <t>2. Hiệu lực báo giá: 30 ngày kể từ ngày báo giá.</t>
+        </is>
+      </c>
+      <c r="B26" s="34" t="n"/>
+      <c r="C26" s="34" t="n"/>
+      <c r="D26" s="34" t="n"/>
+      <c r="E26" s="34" t="n"/>
+      <c r="F26" s="34" t="n"/>
+      <c r="G26" s="34" t="n"/>
+    </row>
+    <row r="27" ht="17.5" customHeight="1">
+      <c r="A27" s="34" t="inlineStr">
+        <is>
+          <t>3. Thời gian giao hàng: trong vòng 03 ngày kể từ khi Quý khách xác nhận đặt hàng.</t>
+        </is>
+      </c>
+      <c r="B27" s="34" t="n"/>
+      <c r="C27" s="34" t="n"/>
+      <c r="D27" s="34" t="n"/>
+      <c r="E27" s="34" t="n"/>
+      <c r="F27" s="34" t="n"/>
+      <c r="G27" s="34" t="n"/>
     </row>
     <row r="28" ht="17.5" customHeight="1">
-      <c r="A28" s="36" t="inlineStr">
-        <is>
-          <t>1. Đơn giá trên đã bao gồm thuế GTGT 8%.</t>
-        </is>
-      </c>
-      <c r="B28" s="36" t="n"/>
-      <c r="C28" s="36" t="n"/>
-      <c r="D28" s="36" t="n"/>
-      <c r="E28" s="36" t="n"/>
-      <c r="F28" s="36" t="n"/>
-      <c r="G28" s="36" t="n"/>
+      <c r="A28" s="34" t="inlineStr">
+        <is>
+          <t>4. Địa điểm giao hàng: tại kho của Quý khách.</t>
+        </is>
+      </c>
+      <c r="B28" s="34" t="n"/>
+      <c r="C28" s="34" t="n"/>
+      <c r="D28" s="34" t="n"/>
+      <c r="E28" s="34" t="n"/>
+      <c r="F28" s="34" t="n"/>
+      <c r="G28" s="34" t="n"/>
     </row>
     <row r="29" ht="17.5" customHeight="1">
-      <c r="A29" s="36" t="inlineStr">
-        <is>
-          <t>2. Hiệu lực báo giá: 30 ngày kể từ ngày báo giá.</t>
-        </is>
-      </c>
-      <c r="B29" s="36" t="n"/>
-      <c r="C29" s="36" t="n"/>
-      <c r="D29" s="36" t="n"/>
-      <c r="E29" s="36" t="n"/>
-      <c r="F29" s="36" t="n"/>
-      <c r="G29" s="36" t="n"/>
-    </row>
-    <row r="30" ht="17.5" customHeight="1">
-      <c r="A30" s="36" t="inlineStr">
-        <is>
-          <t>3. Thời gian giao hàng: trong vòng 03 ngày kể từ khi Quý khách xác nhận đặt hàng.</t>
-        </is>
-      </c>
-      <c r="B30" s="36" t="n"/>
-      <c r="C30" s="36" t="n"/>
-      <c r="D30" s="36" t="n"/>
-      <c r="E30" s="36" t="n"/>
-      <c r="F30" s="36" t="n"/>
-      <c r="G30" s="36" t="n"/>
-    </row>
-    <row r="31" ht="17.5" customHeight="1">
-      <c r="A31" s="36" t="inlineStr">
-        <is>
-          <t>4. Địa điểm giao hàng: tại kho của Quý khách.</t>
-        </is>
-      </c>
-      <c r="B31" s="36" t="n"/>
-      <c r="C31" s="36" t="n"/>
-      <c r="D31" s="36" t="n"/>
-      <c r="E31" s="36" t="n"/>
-      <c r="F31" s="36" t="n"/>
-      <c r="G31" s="36" t="n"/>
-    </row>
-    <row r="32" ht="17.5" customHeight="1">
-      <c r="A32" s="36" t="inlineStr">
+      <c r="A29" s="34" t="inlineStr">
         <is>
           <t>5. Thanh toán: chuyển khoản, 100% khi nhận hàng.</t>
         </is>
       </c>
-      <c r="B32" s="36" t="n"/>
-      <c r="C32" s="36" t="n"/>
-      <c r="D32" s="36" t="n"/>
-      <c r="E32" s="36" t="n"/>
-      <c r="F32" s="36" t="n"/>
-      <c r="G32" s="36" t="n"/>
-    </row>
-    <row r="33" ht="30" customHeight="1">
-      <c r="A33" s="36" t="inlineStr">
+      <c r="B29" s="34" t="n"/>
+      <c r="C29" s="34" t="n"/>
+      <c r="D29" s="34" t="n"/>
+      <c r="E29" s="34" t="n"/>
+      <c r="F29" s="34" t="n"/>
+      <c r="G29" s="34" t="n"/>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="34" t="inlineStr">
         <is>
           <t>6. Thông tin chuyển khoản: Số TK 1066217478 – Ngân hàng TMCP Ngoại thương Việt Nam (Vietcombank) – Chủ tài khoản: CT TNHH KY THUAT CONG TRINH BLT.</t>
         </is>
       </c>
-      <c r="B33" s="36" t="n"/>
-      <c r="C33" s="36" t="n"/>
-      <c r="D33" s="36" t="n"/>
-      <c r="E33" s="36" t="n"/>
-      <c r="F33" s="36" t="n"/>
-      <c r="G33" s="36" t="n"/>
-    </row>
-    <row r="34" ht="6" customHeight="1"/>
-    <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="16" t="inlineStr">
+      <c r="B30" s="34" t="n"/>
+      <c r="C30" s="34" t="n"/>
+      <c r="D30" s="34" t="n"/>
+      <c r="E30" s="34" t="n"/>
+      <c r="F30" s="34" t="n"/>
+      <c r="G30" s="34" t="n"/>
+    </row>
+    <row r="31" ht="6" customHeight="1"/>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="17" t="inlineStr">
         <is>
           <t>Rất mong nhận được sự hợp tác của Quý khách. Trân trọng!</t>
         </is>
       </c>
-      <c r="B35" s="16" t="n"/>
-      <c r="C35" s="16" t="n"/>
-      <c r="D35" s="16" t="n"/>
-      <c r="E35" s="16" t="n"/>
-      <c r="F35" s="16" t="n"/>
-      <c r="G35" s="16" t="n"/>
-    </row>
-    <row r="36" ht="12" customHeight="1"/>
-    <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="37" t="inlineStr">
+      <c r="B32" s="17" t="n"/>
+      <c r="C32" s="17" t="n"/>
+      <c r="D32" s="17" t="n"/>
+      <c r="E32" s="17" t="n"/>
+      <c r="F32" s="17" t="n"/>
+      <c r="G32" s="17" t="n"/>
+    </row>
+    <row r="33" ht="12" customHeight="1"/>
+    <row r="34" ht="18" customHeight="1">
+      <c r="A34" s="35" t="inlineStr">
         <is>
           <t>XÁC NHẬN CỦA KHÁCH HÀNG</t>
         </is>
       </c>
-      <c r="B37" s="37" t="n"/>
-      <c r="C37" s="37" t="n"/>
-      <c r="E37" s="37" t="inlineStr">
+      <c r="B34" s="35" t="n"/>
+      <c r="C34" s="35" t="n"/>
+      <c r="E34" s="35" t="inlineStr">
         <is>
           <t>GIÁM ĐỐC</t>
         </is>
       </c>
-      <c r="F37" s="37" t="n"/>
-      <c r="G37" s="37" t="n"/>
-    </row>
-    <row r="38" ht="15" customHeight="1">
-      <c r="A38" s="38" t="inlineStr">
+      <c r="F34" s="35" t="n"/>
+      <c r="G34" s="35" t="n"/>
+    </row>
+    <row r="35" ht="15" customHeight="1">
+      <c r="A35" s="36" t="inlineStr">
         <is>
           <t>(Ký, ghi rõ họ tên)</t>
         </is>
       </c>
-      <c r="B38" s="38" t="n"/>
-      <c r="C38" s="38" t="n"/>
-      <c r="E38" s="38" t="inlineStr">
+      <c r="B35" s="36" t="n"/>
+      <c r="C35" s="36" t="n"/>
+      <c r="E35" s="36" t="inlineStr">
         <is>
           <t>(Ký, đóng dấu, ghi rõ họ tên)</t>
         </is>
       </c>
-      <c r="F38" s="38" t="n"/>
-      <c r="G38" s="38" t="n"/>
-    </row>
+      <c r="F35" s="36" t="n"/>
+      <c r="G35" s="36" t="n"/>
+    </row>
+    <row r="36" ht="16" customHeight="1"/>
+    <row r="37" ht="16" customHeight="1"/>
+    <row r="38" ht="16" customHeight="1"/>
     <row r="39" ht="16" customHeight="1"/>
-    <row r="40" ht="16" customHeight="1"/>
-    <row r="41" ht="16" customHeight="1"/>
-    <row r="42" ht="16" customHeight="1"/>
-    <row r="43" ht="20" customHeight="1">
-      <c r="E43" s="39" t="inlineStr">
+    <row r="40" ht="20" customHeight="1">
+      <c r="E40" s="37" t="inlineStr">
         <is>
           <t>HỒ VĂN BÌNH</t>
         </is>
       </c>
-      <c r="F43" s="39" t="n"/>
-      <c r="G43" s="39" t="n"/>
+      <c r="F40" s="37" t="n"/>
+      <c r="G40" s="37" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="35">
     <mergeCell ref="A32:G32"/>
-    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="E10:G10"/>
     <mergeCell ref="E13:G13"/>
-    <mergeCell ref="A17:G17"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A8:G8"/>
-    <mergeCell ref="A37:C37"/>
-    <mergeCell ref="A35:G35"/>
-    <mergeCell ref="B1:G1"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="E34:G34"/>
+    <mergeCell ref="E9:G9"/>
+    <mergeCell ref="E40:G40"/>
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A12:C12"/>
-    <mergeCell ref="E15:G15"/>
     <mergeCell ref="A28:G28"/>
-    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="E2:G2"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="A31:G31"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A24:G24"/>
     <mergeCell ref="A30:G30"/>
-    <mergeCell ref="A38:C38"/>
+    <mergeCell ref="A15:G15"/>
+    <mergeCell ref="A35:C35"/>
+    <mergeCell ref="A10:C10"/>
+    <mergeCell ref="A21:E21"/>
     <mergeCell ref="A13:C13"/>
-    <mergeCell ref="E37:G37"/>
-    <mergeCell ref="B4:G4"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="A9:C9"/>
     <mergeCell ref="E12:G12"/>
-    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="E3:G3"/>
     <mergeCell ref="A25:G25"/>
-    <mergeCell ref="A15:C15"/>
-    <mergeCell ref="E43:G43"/>
-    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="B3:D3"/>
     <mergeCell ref="A11:C11"/>
-    <mergeCell ref="E14:G14"/>
     <mergeCell ref="A27:G27"/>
-    <mergeCell ref="A33:G33"/>
-    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="E5:G5"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="E35:G35"/>
+    <mergeCell ref="E4:G4"/>
+    <mergeCell ref="B2:D2"/>
+    <mergeCell ref="E1:G1"/>
   </mergeCells>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.4" right="0.4" top="0.45" bottom="0.6" header="0.5" footer="0.25"/>

</xml_diff>